<commit_message>
Add check for Chandra
</commit_message>
<xml_diff>
--- a/2-multi-document-abbyy-vs-tiled3x2+docparse-paddleocr-paddlevl/test-results/page-level-excels/oocihm.22250/oocihm.22250.1.xlsx
+++ b/2-multi-document-abbyy-vs-tiled3x2+docparse-paddleocr-paddlevl/test-results/page-level-excels/oocihm.22250/oocihm.22250.1.xlsx
@@ -416,14 +416,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y26"/>
+  <dimension ref="A1:Y29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="33" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="35" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
@@ -431,7 +431,7 @@
     <col width="60" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
     <col width="32" customWidth="1" min="12" max="12"/>
-    <col width="31" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
     <col width="60" customWidth="1" min="14" max="14"/>
     <col width="59" customWidth="1" min="15" max="15"/>
     <col width="31" customWidth="1" min="16" max="16"/>
@@ -609,16 +609,20 @@
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
-          <t>L3: stray/suspicious non-ASCII glyph(s): U+00AD SOFT HYPHEN, U+00A6 BROKEN BAR :: è­¦ çƒ‚</t>
+          <t>L3: stray/suspicious non-ASCII glyph(s): U+8B66 CJK UNIFIED IDEOGRAPH-8B66, U+70C2 CJK UNIFIED IDEOGRAPH-70C2 :: 警 烂</t>
         </is>
       </c>
       <c r="K2" s="1" t="inlineStr">
         <is>
-          <t>L12: stray/suspicious non-ASCII glyph(s): U+20AC EURO SIGN :: â€” = _ =</t>
+          <t>L1: BOM/control character at start of file | stray/suspicious non-ASCII glyph(s): U+FEFF ZERO WIDTH NO-BREAK SPACE :: [BOM]IMAGE EVALUATION</t>
         </is>
       </c>
       <c r="L2" s="1" t="inlineStr"/>
-      <c r="M2" s="1" t="inlineStr"/>
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>L1: BOM/control character at start of file | stray/suspicious non-ASCII glyph(s): U+FEFF ZERO WIDTH NO-BREAK SPACE :: [BOM]IMAGE EVALUATION</t>
+        </is>
+      </c>
       <c r="N2" s="1" t="inlineStr">
         <is>
           <t>L8: isolated marker/symbol line :: 45</t>
@@ -657,7 +661,7 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr"/>
@@ -672,12 +676,12 @@
       </c>
       <c r="J3" s="1" t="inlineStr">
         <is>
-          <t>L29: stray/suspicious non-ASCII glyph(s): U+20AC EURO SIGN :: 6 â€³</t>
+          <t>L22: stray/suspicious non-ASCII glyph(s): U+5FC3 CJK UNIFIED IDEOGRAPH-5FC3 | isolated marker/symbol line :: 心</t>
         </is>
       </c>
       <c r="K3" s="1" t="inlineStr">
         <is>
-          <t>L14: stray/suspicious non-ASCII glyph(s): U+20AC EURO SIGN, U+00A2 CENT SIGN :: Hâ€¢ MAS</t>
+          <t>L14: stray/suspicious non-ASCII glyph(s): U+2022 BULLET :: H• MAS</t>
         </is>
       </c>
       <c r="L3" s="1" t="inlineStr"/>
@@ -689,7 +693,7 @@
       </c>
       <c r="O3" s="1" t="inlineStr">
         <is>
-          <t>L19: isolated marker/symbol line :: 6"</t>
+          <t>L12: symbol-only separator/garbage line :: — = _ =</t>
         </is>
       </c>
       <c r="P3" s="1" t="inlineStr"/>
@@ -727,7 +731,7 @@
       <c r="I4" s="1" t="inlineStr"/>
       <c r="J4" s="1" t="inlineStr">
         <is>
-          <t>L44: stray/suspicious non-ASCII glyph(s): U+20AC EURO SIGN | isolated marker/symbol line :: ã€‚</t>
+          <t>L35: stray/suspicious non-ASCII glyph(s): U+4E8C CJK UNIFIED IDEOGRAPH-4E8C | isolated marker/symbol line :: 二</t>
         </is>
       </c>
       <c r="K4" s="1" t="inlineStr"/>
@@ -740,7 +744,7 @@
       </c>
       <c r="O4" s="1" t="inlineStr">
         <is>
-          <t>L30: symbol-only separator/garbage line :: (716) 872-4503</t>
+          <t>L19: isolated marker/symbol line :: 6"</t>
         </is>
       </c>
       <c r="P4" s="1" t="inlineStr"/>
@@ -762,12 +766,12 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>31</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr"/>
@@ -776,7 +780,11 @@
       <c r="G5" s="1" t="inlineStr"/>
       <c r="H5" s="1" t="inlineStr"/>
       <c r="I5" s="1" t="inlineStr"/>
-      <c r="J5" s="1" t="inlineStr"/>
+      <c r="J5" s="1" t="inlineStr">
+        <is>
+          <t>L40: stray/suspicious non-ASCII glyph(s): U+7ACB CJK UNIFIED IDEOGRAPH-7ACB | isolated marker/symbol line :: 立</t>
+        </is>
+      </c>
       <c r="K5" s="1" t="inlineStr"/>
       <c r="L5" s="1" t="inlineStr"/>
       <c r="M5" s="1" t="inlineStr"/>
@@ -785,7 +793,11 @@
           <t>L11: symbol-only separator/garbage line :: 1.0</t>
         </is>
       </c>
-      <c r="O5" s="1" t="inlineStr"/>
+      <c r="O5" s="1" t="inlineStr">
+        <is>
+          <t>L30: symbol-only separator/garbage line :: (716) 872-4503</t>
+        </is>
+      </c>
       <c r="P5" s="1" t="inlineStr"/>
       <c r="Q5" s="1" t="inlineStr"/>
       <c r="R5" s="1" t="inlineStr"/>
@@ -819,7 +831,11 @@
       <c r="G6" s="1" t="inlineStr"/>
       <c r="H6" s="1" t="inlineStr"/>
       <c r="I6" s="1" t="inlineStr"/>
-      <c r="J6" s="1" t="inlineStr"/>
+      <c r="J6" s="1" t="inlineStr">
+        <is>
+          <t>L44: stray/suspicious non-ASCII glyph(s): U+3002 IDEOGRAPHIC FULL STOP | isolated marker/symbol line :: 。</t>
+        </is>
+      </c>
       <c r="K6" s="1" t="inlineStr"/>
       <c r="L6" s="1" t="inlineStr"/>
       <c r="M6" s="1" t="inlineStr"/>
@@ -977,7 +993,7 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr">
@@ -1025,7 +1041,7 @@
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D11" s="1" t="inlineStr"/>
@@ -1063,12 +1079,12 @@
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>28</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D12" s="1" t="inlineStr"/>
@@ -1255,7 +1271,7 @@
       <c r="M16" s="1" t="inlineStr"/>
       <c r="N16" s="1" t="inlineStr">
         <is>
-          <t>L23: isolated marker/symbol line :: U</t>
+          <t>L22: stray/suspicious non-ASCII glyph(s): U+5FC3 CJK UNIFIED IDEOGRAPH-5FC3 | isolated marker/symbol line :: 心</t>
         </is>
       </c>
       <c r="O16" s="1" t="inlineStr"/>
@@ -1298,7 +1314,7 @@
       <c r="M17" s="1" t="inlineStr"/>
       <c r="N17" s="1" t="inlineStr">
         <is>
-          <t>L24: symbol-only separator/garbage line :: 1.8</t>
+          <t>L23: isolated marker/symbol line :: U</t>
         </is>
       </c>
       <c r="O17" s="1" t="inlineStr"/>
@@ -1329,7 +1345,7 @@
       <c r="M18" s="1" t="inlineStr"/>
       <c r="N18" s="1" t="inlineStr">
         <is>
-          <t>L25: symbol-only separator/garbage line :: 111.25</t>
+          <t>L24: symbol-only separator/garbage line :: 1.8</t>
         </is>
       </c>
       <c r="O18" s="1" t="inlineStr"/>
@@ -1360,7 +1376,7 @@
       <c r="M19" s="1" t="inlineStr"/>
       <c r="N19" s="1" t="inlineStr">
         <is>
-          <t>L26: symbol-only separator/garbage line :: 1.4</t>
+          <t>L25: symbol-only separator/garbage line :: 111.25</t>
         </is>
       </c>
       <c r="O19" s="1" t="inlineStr"/>
@@ -1391,7 +1407,7 @@
       <c r="M20" s="1" t="inlineStr"/>
       <c r="N20" s="1" t="inlineStr">
         <is>
-          <t>L27: symbol-only separator/garbage line :: 1.6</t>
+          <t>L26: symbol-only separator/garbage line :: 1.4</t>
         </is>
       </c>
       <c r="O20" s="1" t="inlineStr"/>
@@ -1422,7 +1438,7 @@
       <c r="M21" s="1" t="inlineStr"/>
       <c r="N21" s="1" t="inlineStr">
         <is>
-          <t>L28: isolated marker/symbol line :: D</t>
+          <t>L27: symbol-only separator/garbage line :: 1.6</t>
         </is>
       </c>
       <c r="O21" s="1" t="inlineStr"/>
@@ -1453,7 +1469,7 @@
       <c r="M22" s="1" t="inlineStr"/>
       <c r="N22" s="1" t="inlineStr">
         <is>
-          <t>L34: isolated marker/symbol line :: =</t>
+          <t>L28: isolated marker/symbol line :: D</t>
         </is>
       </c>
       <c r="O22" s="1" t="inlineStr"/>
@@ -1484,7 +1500,7 @@
       <c r="M23" s="1" t="inlineStr"/>
       <c r="N23" s="1" t="inlineStr">
         <is>
-          <t>L36: isolated marker/symbol line :: T</t>
+          <t>L29: isolated marker/symbol line :: 6 ″</t>
         </is>
       </c>
       <c r="O23" s="1" t="inlineStr"/>
@@ -1515,7 +1531,7 @@
       <c r="M24" s="1" t="inlineStr"/>
       <c r="N24" s="1" t="inlineStr">
         <is>
-          <t>L39: symbol-only separator/garbage line :: (716) 872-4503</t>
+          <t>L34: isolated marker/symbol line :: =</t>
         </is>
       </c>
       <c r="O24" s="1" t="inlineStr"/>
@@ -1546,7 +1562,7 @@
       <c r="M25" s="1" t="inlineStr"/>
       <c r="N25" s="1" t="inlineStr">
         <is>
-          <t>L40: isolated marker/symbol line :: ç«‹</t>
+          <t>L35: stray/suspicious non-ASCII glyph(s): U+4E8C CJK UNIFIED IDEOGRAPH-4E8C | isolated marker/symbol line :: 二</t>
         </is>
       </c>
       <c r="O25" s="1" t="inlineStr"/>
@@ -1577,7 +1593,7 @@
       <c r="M26" s="1" t="inlineStr"/>
       <c r="N26" s="1" t="inlineStr">
         <is>
-          <t>L44: stray/suspicious non-ASCII glyph(s): U+20AC EURO SIGN | isolated marker/symbol line :: ã€‚</t>
+          <t>L36: isolated marker/symbol line :: T</t>
         </is>
       </c>
       <c r="O26" s="1" t="inlineStr"/>
@@ -1592,6 +1608,99 @@
       <c r="X26" s="1" t="inlineStr"/>
       <c r="Y26" s="1" t="inlineStr"/>
     </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr"/>
+      <c r="B27" s="1" t="inlineStr"/>
+      <c r="C27" s="1" t="inlineStr"/>
+      <c r="D27" s="1" t="inlineStr"/>
+      <c r="E27" s="1" t="inlineStr"/>
+      <c r="F27" s="1" t="inlineStr"/>
+      <c r="G27" s="1" t="inlineStr"/>
+      <c r="H27" s="1" t="inlineStr"/>
+      <c r="I27" s="1" t="inlineStr"/>
+      <c r="J27" s="1" t="inlineStr"/>
+      <c r="K27" s="1" t="inlineStr"/>
+      <c r="L27" s="1" t="inlineStr"/>
+      <c r="M27" s="1" t="inlineStr"/>
+      <c r="N27" s="1" t="inlineStr">
+        <is>
+          <t>L39: symbol-only separator/garbage line :: (716) 872-4503</t>
+        </is>
+      </c>
+      <c r="O27" s="1" t="inlineStr"/>
+      <c r="P27" s="1" t="inlineStr"/>
+      <c r="Q27" s="1" t="inlineStr"/>
+      <c r="R27" s="1" t="inlineStr"/>
+      <c r="S27" s="1" t="inlineStr"/>
+      <c r="T27" s="1" t="inlineStr"/>
+      <c r="U27" s="1" t="inlineStr"/>
+      <c r="V27" s="1" t="inlineStr"/>
+      <c r="W27" s="1" t="inlineStr"/>
+      <c r="X27" s="1" t="inlineStr"/>
+      <c r="Y27" s="1" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr"/>
+      <c r="B28" s="1" t="inlineStr"/>
+      <c r="C28" s="1" t="inlineStr"/>
+      <c r="D28" s="1" t="inlineStr"/>
+      <c r="E28" s="1" t="inlineStr"/>
+      <c r="F28" s="1" t="inlineStr"/>
+      <c r="G28" s="1" t="inlineStr"/>
+      <c r="H28" s="1" t="inlineStr"/>
+      <c r="I28" s="1" t="inlineStr"/>
+      <c r="J28" s="1" t="inlineStr"/>
+      <c r="K28" s="1" t="inlineStr"/>
+      <c r="L28" s="1" t="inlineStr"/>
+      <c r="M28" s="1" t="inlineStr"/>
+      <c r="N28" s="1" t="inlineStr">
+        <is>
+          <t>L40: stray/suspicious non-ASCII glyph(s): U+7ACB CJK UNIFIED IDEOGRAPH-7ACB | isolated marker/symbol line :: 立</t>
+        </is>
+      </c>
+      <c r="O28" s="1" t="inlineStr"/>
+      <c r="P28" s="1" t="inlineStr"/>
+      <c r="Q28" s="1" t="inlineStr"/>
+      <c r="R28" s="1" t="inlineStr"/>
+      <c r="S28" s="1" t="inlineStr"/>
+      <c r="T28" s="1" t="inlineStr"/>
+      <c r="U28" s="1" t="inlineStr"/>
+      <c r="V28" s="1" t="inlineStr"/>
+      <c r="W28" s="1" t="inlineStr"/>
+      <c r="X28" s="1" t="inlineStr"/>
+      <c r="Y28" s="1" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr"/>
+      <c r="B29" s="1" t="inlineStr"/>
+      <c r="C29" s="1" t="inlineStr"/>
+      <c r="D29" s="1" t="inlineStr"/>
+      <c r="E29" s="1" t="inlineStr"/>
+      <c r="F29" s="1" t="inlineStr"/>
+      <c r="G29" s="1" t="inlineStr"/>
+      <c r="H29" s="1" t="inlineStr"/>
+      <c r="I29" s="1" t="inlineStr"/>
+      <c r="J29" s="1" t="inlineStr"/>
+      <c r="K29" s="1" t="inlineStr"/>
+      <c r="L29" s="1" t="inlineStr"/>
+      <c r="M29" s="1" t="inlineStr"/>
+      <c r="N29" s="1" t="inlineStr">
+        <is>
+          <t>L44: stray/suspicious non-ASCII glyph(s): U+3002 IDEOGRAPHIC FULL STOP | isolated marker/symbol line :: 。</t>
+        </is>
+      </c>
+      <c r="O29" s="1" t="inlineStr"/>
+      <c r="P29" s="1" t="inlineStr"/>
+      <c r="Q29" s="1" t="inlineStr"/>
+      <c r="R29" s="1" t="inlineStr"/>
+      <c r="S29" s="1" t="inlineStr"/>
+      <c r="T29" s="1" t="inlineStr"/>
+      <c r="U29" s="1" t="inlineStr"/>
+      <c r="V29" s="1" t="inlineStr"/>
+      <c r="W29" s="1" t="inlineStr"/>
+      <c r="X29" s="1" t="inlineStr"/>
+      <c r="Y29" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>